<commit_message>
Fixed production files and added BOM.csv in BOMs folder and root folder
</commit_message>
<xml_diff>
--- a/BOMs/BOM_ORDER.xlsx
+++ b/BOMs/BOM_ORDER.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Simon\Documents\KiCad\desings\4_DMX node\BOMs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{05D89962-65B0-4B14-ACEA-DC485BF0AB54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1372D22A-C904-4495-93E3-8CAF3AB35CBA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" xr2:uid="{9B84EF14-36DD-40E4-AAD2-543AD15C4A8A}"/>
   </bookViews>
@@ -70,7 +70,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2047" uniqueCount="655">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2055" uniqueCount="663">
   <si>
     <t>Id</t>
   </si>
@@ -2035,6 +2035,30 @@
   </si>
   <si>
     <t>https://www.tinytronics.nl/en/power/batteries/li-po/pkcell-li-po-battery-3.7v-2000mah-jst-ph-lp803860</t>
+  </si>
+  <si>
+    <t>shipping LCSC</t>
+  </si>
+  <si>
+    <t>Shipping JLCPCB</t>
+  </si>
+  <si>
+    <t>Shipping Tinytronics</t>
+  </si>
+  <si>
+    <t>Shipping Mouser</t>
+  </si>
+  <si>
+    <t>Total</t>
+  </si>
+  <si>
+    <t>JLCPCB Main PCB inc. Stencil</t>
+  </si>
+  <si>
+    <t>JLCPCB WIFI PCB inc. Stencil</t>
+  </si>
+  <si>
+    <t>JLCPCB Display PCB inc. Stencil</t>
   </si>
 </sst>
 </file>
@@ -2142,7 +2166,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -2193,10 +2217,11 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="3" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="44" fontId="8" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="44" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Currency" xfId="1" builtinId="4"/>
@@ -2204,139 +2229,7 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 2" xfId="2" xr:uid="{B5D1B2ED-513F-44B5-BB21-F052053D13F4}"/>
   </cellStyles>
-  <dxfs count="128">
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color indexed="12"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <alignment textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color indexed="12"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <alignment textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color indexed="12"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <alignment textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="122">
     <dxf>
       <fill>
         <patternFill>
@@ -2419,6 +2312,36 @@
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color indexed="12"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <alignment textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
@@ -2657,6 +2580,36 @@
     </dxf>
     <dxf>
       <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color indexed="12"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <alignment textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <font>
         <b val="0"/>
         <strike val="0"/>
         <outline val="0"/>
@@ -2887,6 +2840,36 @@
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color indexed="12"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <alignment textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
@@ -3316,25 +3299,25 @@
   </dxfs>
   <tableStyles count="2" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16">
     <tableStyle name="TableStylePreset3_Accent1" pivot="0" count="7" xr9:uid="{17788B69-A5A2-442D-970D-4F3F58D2C1D1}">
-      <tableStyleElement type="wholeTable" dxfId="127"/>
-      <tableStyleElement type="headerRow" dxfId="126"/>
-      <tableStyleElement type="totalRow" dxfId="125"/>
-      <tableStyleElement type="firstColumn" dxfId="124"/>
-      <tableStyleElement type="lastColumn" dxfId="123"/>
-      <tableStyleElement type="firstRowStripe" dxfId="122"/>
-      <tableStyleElement type="firstColumnStripe" dxfId="121"/>
+      <tableStyleElement type="wholeTable" dxfId="121"/>
+      <tableStyleElement type="headerRow" dxfId="120"/>
+      <tableStyleElement type="totalRow" dxfId="119"/>
+      <tableStyleElement type="firstColumn" dxfId="118"/>
+      <tableStyleElement type="lastColumn" dxfId="117"/>
+      <tableStyleElement type="firstRowStripe" dxfId="116"/>
+      <tableStyleElement type="firstColumnStripe" dxfId="115"/>
     </tableStyle>
     <tableStyle name="PivotStylePreset2_Accent1" table="0" count="10" xr9:uid="{49D30C32-15C7-40F8-9F26-4D109DA1EB3E}">
-      <tableStyleElement type="headerRow" dxfId="120"/>
-      <tableStyleElement type="totalRow" dxfId="119"/>
-      <tableStyleElement type="firstRowStripe" dxfId="118"/>
-      <tableStyleElement type="firstColumnStripe" dxfId="117"/>
-      <tableStyleElement type="firstSubtotalRow" dxfId="116"/>
-      <tableStyleElement type="secondSubtotalRow" dxfId="115"/>
-      <tableStyleElement type="firstRowSubheading" dxfId="114"/>
-      <tableStyleElement type="secondRowSubheading" dxfId="113"/>
-      <tableStyleElement type="pageFieldLabels" dxfId="112"/>
-      <tableStyleElement type="pageFieldValues" dxfId="111"/>
+      <tableStyleElement type="headerRow" dxfId="114"/>
+      <tableStyleElement type="totalRow" dxfId="113"/>
+      <tableStyleElement type="firstRowStripe" dxfId="112"/>
+      <tableStyleElement type="firstColumnStripe" dxfId="111"/>
+      <tableStyleElement type="firstSubtotalRow" dxfId="110"/>
+      <tableStyleElement type="secondSubtotalRow" dxfId="109"/>
+      <tableStyleElement type="firstRowSubheading" dxfId="108"/>
+      <tableStyleElement type="secondRowSubheading" dxfId="107"/>
+      <tableStyleElement type="pageFieldLabels" dxfId="106"/>
+      <tableStyleElement type="pageFieldValues" dxfId="105"/>
     </tableStyle>
   </tableStyles>
   <extLst>
@@ -3524,36 +3507,36 @@
   </sortState>
   <tableColumns count="29">
     <tableColumn id="1" xr3:uid="{193D4942-D9C7-4808-9664-ED233B7BC77F}" uniqueName="1" name="Id" queryTableFieldId="1"/>
-    <tableColumn id="2" xr3:uid="{EBE99961-81FC-436F-B8F4-C920E55866B1}" uniqueName="2" name="Designator" queryTableFieldId="2" dataDxfId="110"/>
-    <tableColumn id="3" xr3:uid="{68D5AD26-CBA6-4EC2-A9F1-D603B2F6AF06}" uniqueName="3" name="Footprint" queryTableFieldId="3" dataDxfId="109"/>
+    <tableColumn id="2" xr3:uid="{EBE99961-81FC-436F-B8F4-C920E55866B1}" uniqueName="2" name="Designator" queryTableFieldId="2" dataDxfId="104"/>
+    <tableColumn id="3" xr3:uid="{68D5AD26-CBA6-4EC2-A9F1-D603B2F6AF06}" uniqueName="3" name="Footprint" queryTableFieldId="3" dataDxfId="103"/>
     <tableColumn id="4" xr3:uid="{C69663E0-3934-402E-A217-B04C029903F9}" uniqueName="4" name="Quantity" queryTableFieldId="4"/>
-    <tableColumn id="5" xr3:uid="{EFC1BF42-A0F8-4167-A78B-971913DD5EC6}" uniqueName="5" name="Designation" queryTableFieldId="5" dataDxfId="108"/>
-    <tableColumn id="6" xr3:uid="{ADFEF14D-AB5A-4337-BFD4-9F22C06A037A}" uniqueName="6" name="Supplier and ref" queryTableFieldId="6" dataDxfId="107"/>
-    <tableColumn id="7" xr3:uid="{5FF69B16-46E7-4D4B-92E4-918E69492B30}" uniqueName="7" name="Column1" queryTableFieldId="7" dataDxfId="106"/>
-    <tableColumn id="10" xr3:uid="{7ECCF4D2-A4BB-4FB1-AB47-D80526DE1596}" uniqueName="10" name="Needed quantity" queryTableFieldId="9" dataDxfId="105">
+    <tableColumn id="5" xr3:uid="{EFC1BF42-A0F8-4167-A78B-971913DD5EC6}" uniqueName="5" name="Designation" queryTableFieldId="5" dataDxfId="102"/>
+    <tableColumn id="6" xr3:uid="{ADFEF14D-AB5A-4337-BFD4-9F22C06A037A}" uniqueName="6" name="Supplier and ref" queryTableFieldId="6" dataDxfId="101"/>
+    <tableColumn id="7" xr3:uid="{5FF69B16-46E7-4D4B-92E4-918E69492B30}" uniqueName="7" name="Column1" queryTableFieldId="7" dataDxfId="100"/>
+    <tableColumn id="10" xr3:uid="{7ECCF4D2-A4BB-4FB1-AB47-D80526DE1596}" uniqueName="10" name="Needed quantity" queryTableFieldId="9" dataDxfId="99">
       <calculatedColumnFormula>2*Artnet_DMX_Converter5[[#This Row],[Quantity]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{B90649C3-9530-44F6-9F83-0F46EA369F24}" uniqueName="8" name="-" queryTableFieldId="8" dataDxfId="104"/>
-    <tableColumn id="11" xr3:uid="{8BB3B2CB-709B-40DE-91FE-851022C724E2}" uniqueName="11" name="LCSC" queryTableFieldId="10" dataDxfId="103"/>
-    <tableColumn id="12" xr3:uid="{5B21BDC3-D99E-43DA-A2E4-B05F14DDA14D}" uniqueName="12" name="MOUSER" queryTableFieldId="11" dataDxfId="102"/>
-    <tableColumn id="13" xr3:uid="{B0CDCEBA-8AC4-4942-9413-2D530A7F2761}" uniqueName="13" name="Already in another pcb" queryTableFieldId="12" dataDxfId="101"/>
-    <tableColumn id="14" xr3:uid="{8340A12D-F318-4D9C-969B-3117A5EADB1A}" uniqueName="14" name="Enough?" queryTableFieldId="13" dataDxfId="100"/>
-    <tableColumn id="15" xr3:uid="{1ED5A8A2-1611-49FA-A788-90397B1162E3}" uniqueName="15" name="Mrf#" queryTableFieldId="14" dataDxfId="99"/>
-    <tableColumn id="16" xr3:uid="{07C56306-EF8D-45EF-BC0C-FA7F2A15FEF3}" uniqueName="16" name="Mfr." queryTableFieldId="15" dataDxfId="98"/>
-    <tableColumn id="17" xr3:uid="{19635C0F-7BD1-4660-98C6-93346F766B86}" uniqueName="17" name="Order Qty." queryTableFieldId="16" dataDxfId="97" dataCellStyle="Currency"/>
-    <tableColumn id="18" xr3:uid="{A46DB81F-05A4-4B42-8CA7-8DD56227E5E7}" uniqueName="18" name="Unit Price(USD)" queryTableFieldId="17" dataDxfId="96" dataCellStyle="Currency"/>
-    <tableColumn id="19" xr3:uid="{570EBF30-7625-4C4F-A1A9-5A6C29E3344C}" uniqueName="19" name="Ext.Price(USD)" queryTableFieldId="18" dataDxfId="95" dataCellStyle="Currency"/>
-    <tableColumn id="20" xr3:uid="{1210C2A8-B78E-4F49-8D59-4D7358DDF469}" uniqueName="20" name="LCSC#/MOUSER" queryTableFieldId="19" dataDxfId="94"/>
-    <tableColumn id="21" xr3:uid="{DCDFBA0B-E1DF-4891-B6DE-50DD37843C8F}" uniqueName="21" name="Package" queryTableFieldId="20" dataDxfId="93"/>
-    <tableColumn id="22" xr3:uid="{EE553BAA-235A-4ADE-BF21-5A6D487E525F}" uniqueName="22" name="Min" queryTableFieldId="21" dataDxfId="92"/>
-    <tableColumn id="23" xr3:uid="{EF5D702D-6003-4207-8949-2FAAAEA59C21}" uniqueName="23" name="Mult" queryTableFieldId="22" dataDxfId="91"/>
-    <tableColumn id="24" xr3:uid="{FC548331-4E82-4F18-8F1B-96AD5CFD679F}" uniqueName="24" name="SPQ" queryTableFieldId="23" dataDxfId="90"/>
-    <tableColumn id="25" xr3:uid="{4CE5E4B3-AC89-4D44-992B-1F594AE2EC4A}" uniqueName="25" name="Availability" queryTableFieldId="24" dataDxfId="89"/>
-    <tableColumn id="26" xr3:uid="{8719B838-3310-4B06-B6C2-7223B1B40BC9}" uniqueName="26" name="Stock Status" queryTableFieldId="25" dataDxfId="88"/>
-    <tableColumn id="27" xr3:uid="{2577FF1C-2965-441F-B3FF-7C6FD0944441}" uniqueName="27" name="Customer Notes" queryTableFieldId="26" dataDxfId="87"/>
-    <tableColumn id="28" xr3:uid="{5613E865-76FA-42C7-807E-255777292765}" uniqueName="28" name="Description" queryTableFieldId="27" dataDxfId="86"/>
-    <tableColumn id="29" xr3:uid="{DC4F61A6-52E4-4ABC-BD2A-0891230BC00B}" uniqueName="29" name="Matched status" queryTableFieldId="28" dataDxfId="5"/>
-    <tableColumn id="30" xr3:uid="{F1A13F5D-E76A-4CC6-B004-7EA2E6343DD2}" uniqueName="30" name="Product Link" queryTableFieldId="29" dataDxfId="4" dataCellStyle="Hyperlink 2"/>
+    <tableColumn id="8" xr3:uid="{B90649C3-9530-44F6-9F83-0F46EA369F24}" uniqueName="8" name="-" queryTableFieldId="8" dataDxfId="98"/>
+    <tableColumn id="11" xr3:uid="{8BB3B2CB-709B-40DE-91FE-851022C724E2}" uniqueName="11" name="LCSC" queryTableFieldId="10" dataDxfId="97"/>
+    <tableColumn id="12" xr3:uid="{5B21BDC3-D99E-43DA-A2E4-B05F14DDA14D}" uniqueName="12" name="MOUSER" queryTableFieldId="11" dataDxfId="96"/>
+    <tableColumn id="13" xr3:uid="{B0CDCEBA-8AC4-4942-9413-2D530A7F2761}" uniqueName="13" name="Already in another pcb" queryTableFieldId="12" dataDxfId="95"/>
+    <tableColumn id="14" xr3:uid="{8340A12D-F318-4D9C-969B-3117A5EADB1A}" uniqueName="14" name="Enough?" queryTableFieldId="13" dataDxfId="94"/>
+    <tableColumn id="15" xr3:uid="{1ED5A8A2-1611-49FA-A788-90397B1162E3}" uniqueName="15" name="Mrf#" queryTableFieldId="14" dataDxfId="93"/>
+    <tableColumn id="16" xr3:uid="{07C56306-EF8D-45EF-BC0C-FA7F2A15FEF3}" uniqueName="16" name="Mfr." queryTableFieldId="15" dataDxfId="92"/>
+    <tableColumn id="17" xr3:uid="{19635C0F-7BD1-4660-98C6-93346F766B86}" uniqueName="17" name="Order Qty." queryTableFieldId="16" dataDxfId="91" dataCellStyle="Currency"/>
+    <tableColumn id="18" xr3:uid="{A46DB81F-05A4-4B42-8CA7-8DD56227E5E7}" uniqueName="18" name="Unit Price(USD)" queryTableFieldId="17" dataDxfId="90" dataCellStyle="Currency"/>
+    <tableColumn id="19" xr3:uid="{570EBF30-7625-4C4F-A1A9-5A6C29E3344C}" uniqueName="19" name="Ext.Price(USD)" queryTableFieldId="18" dataDxfId="89" dataCellStyle="Currency"/>
+    <tableColumn id="20" xr3:uid="{1210C2A8-B78E-4F49-8D59-4D7358DDF469}" uniqueName="20" name="LCSC#/MOUSER" queryTableFieldId="19" dataDxfId="88"/>
+    <tableColumn id="21" xr3:uid="{DCDFBA0B-E1DF-4891-B6DE-50DD37843C8F}" uniqueName="21" name="Package" queryTableFieldId="20" dataDxfId="87"/>
+    <tableColumn id="22" xr3:uid="{EE553BAA-235A-4ADE-BF21-5A6D487E525F}" uniqueName="22" name="Min" queryTableFieldId="21" dataDxfId="86"/>
+    <tableColumn id="23" xr3:uid="{EF5D702D-6003-4207-8949-2FAAAEA59C21}" uniqueName="23" name="Mult" queryTableFieldId="22" dataDxfId="85"/>
+    <tableColumn id="24" xr3:uid="{FC548331-4E82-4F18-8F1B-96AD5CFD679F}" uniqueName="24" name="SPQ" queryTableFieldId="23" dataDxfId="84"/>
+    <tableColumn id="25" xr3:uid="{4CE5E4B3-AC89-4D44-992B-1F594AE2EC4A}" uniqueName="25" name="Availability" queryTableFieldId="24" dataDxfId="83"/>
+    <tableColumn id="26" xr3:uid="{8719B838-3310-4B06-B6C2-7223B1B40BC9}" uniqueName="26" name="Stock Status" queryTableFieldId="25" dataDxfId="82"/>
+    <tableColumn id="27" xr3:uid="{2577FF1C-2965-441F-B3FF-7C6FD0944441}" uniqueName="27" name="Customer Notes" queryTableFieldId="26" dataDxfId="81"/>
+    <tableColumn id="28" xr3:uid="{5613E865-76FA-42C7-807E-255777292765}" uniqueName="28" name="Description" queryTableFieldId="27" dataDxfId="80"/>
+    <tableColumn id="29" xr3:uid="{DC4F61A6-52E4-4ABC-BD2A-0891230BC00B}" uniqueName="29" name="Matched status" queryTableFieldId="28" dataDxfId="79"/>
+    <tableColumn id="30" xr3:uid="{F1A13F5D-E76A-4CC6-B004-7EA2E6343DD2}" uniqueName="30" name="Product Link" queryTableFieldId="29" dataDxfId="78" dataCellStyle="Hyperlink 2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -3567,36 +3550,36 @@
   </sortState>
   <tableColumns count="29">
     <tableColumn id="1" xr3:uid="{497A9602-423A-4EE5-A4C3-05DBCE27F0C5}" uniqueName="1" name="Id" queryTableFieldId="1"/>
-    <tableColumn id="2" xr3:uid="{248C9EEE-C317-4CF2-8FF9-EBC3B367C080}" uniqueName="2" name="Designator" queryTableFieldId="2" dataDxfId="85"/>
-    <tableColumn id="3" xr3:uid="{36AFF123-E529-4AD9-B586-671130A051FA}" uniqueName="3" name="Footprint" queryTableFieldId="3" dataDxfId="84"/>
+    <tableColumn id="2" xr3:uid="{248C9EEE-C317-4CF2-8FF9-EBC3B367C080}" uniqueName="2" name="Designator" queryTableFieldId="2" dataDxfId="77"/>
+    <tableColumn id="3" xr3:uid="{36AFF123-E529-4AD9-B586-671130A051FA}" uniqueName="3" name="Footprint" queryTableFieldId="3" dataDxfId="76"/>
     <tableColumn id="4" xr3:uid="{3676B207-F980-400C-B584-7AEC2C881662}" uniqueName="4" name="Quantity" queryTableFieldId="4"/>
-    <tableColumn id="5" xr3:uid="{5E97CF41-ABB3-47AE-A0AC-B0E7E29D04F2}" uniqueName="5" name="Designation" queryTableFieldId="5" dataDxfId="83"/>
-    <tableColumn id="6" xr3:uid="{9E4029D5-EC40-4FD8-A618-F86B9AC55CCF}" uniqueName="6" name="Supplier and ref" queryTableFieldId="6" dataDxfId="82"/>
-    <tableColumn id="7" xr3:uid="{AD3BD5D5-70CF-457B-9E36-2BF3A5A4569F}" uniqueName="7" name="Column1" queryTableFieldId="7" dataDxfId="81"/>
-    <tableColumn id="8" xr3:uid="{312509E5-FBDF-4828-AE6F-FA834B68DF72}" uniqueName="8" name="Needed quantity" queryTableFieldId="8" dataDxfId="80">
+    <tableColumn id="5" xr3:uid="{5E97CF41-ABB3-47AE-A0AC-B0E7E29D04F2}" uniqueName="5" name="Designation" queryTableFieldId="5" dataDxfId="75"/>
+    <tableColumn id="6" xr3:uid="{9E4029D5-EC40-4FD8-A618-F86B9AC55CCF}" uniqueName="6" name="Supplier and ref" queryTableFieldId="6" dataDxfId="74"/>
+    <tableColumn id="7" xr3:uid="{AD3BD5D5-70CF-457B-9E36-2BF3A5A4569F}" uniqueName="7" name="Column1" queryTableFieldId="7" dataDxfId="73"/>
+    <tableColumn id="8" xr3:uid="{312509E5-FBDF-4828-AE6F-FA834B68DF72}" uniqueName="8" name="Needed quantity" queryTableFieldId="8" dataDxfId="72">
       <calculatedColumnFormula>2*Display_panel7[[#This Row],[Quantity]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{466BF7CA-A66E-4E93-A410-26712E4A088D}" uniqueName="9" name="-" queryTableFieldId="9" dataDxfId="79"/>
-    <tableColumn id="10" xr3:uid="{EF9CED38-6BA4-4B5E-A768-E8F7877DA34C}" uniqueName="10" name="LCSC" queryTableFieldId="10" dataDxfId="78"/>
-    <tableColumn id="11" xr3:uid="{B8AF37A0-7622-4CE8-B4F8-07F8A264DAFC}" uniqueName="11" name="MOUSER" queryTableFieldId="11" dataDxfId="77"/>
-    <tableColumn id="12" xr3:uid="{3CC847EE-DB6C-4D10-A4FE-5AF7D6DAC000}" uniqueName="12" name="Already in another pcb" queryTableFieldId="12" dataDxfId="76"/>
-    <tableColumn id="13" xr3:uid="{4209E125-D2D4-4118-AAF7-2424A4EE1570}" uniqueName="13" name="--" queryTableFieldId="13" dataDxfId="75"/>
-    <tableColumn id="14" xr3:uid="{F77F0236-F98A-4965-9182-ADC25F4B7E38}" uniqueName="14" name="Mrf#" queryTableFieldId="14" dataDxfId="74"/>
-    <tableColumn id="15" xr3:uid="{35B8A93E-B4A7-4A83-9024-CC101868A70A}" uniqueName="15" name="Mfr." queryTableFieldId="15" dataDxfId="73"/>
-    <tableColumn id="16" xr3:uid="{E562ACF4-D8CD-4985-8EC9-26D45054BB92}" uniqueName="16" name="Order Qty." queryTableFieldId="16" dataDxfId="72" dataCellStyle="Currency"/>
-    <tableColumn id="17" xr3:uid="{4B8A9EA3-8B9F-48DB-B5CE-DD5C61A296C3}" uniqueName="17" name="Unit Price(USD)" queryTableFieldId="17" dataDxfId="71" dataCellStyle="Currency"/>
-    <tableColumn id="18" xr3:uid="{681F7274-0403-4F56-A317-DD049A8A07BF}" uniqueName="18" name="Ext.Price(USD)" queryTableFieldId="18" dataDxfId="70" dataCellStyle="Currency"/>
-    <tableColumn id="19" xr3:uid="{6073EC40-E9B7-4260-A82D-A28FAFFCC35E}" uniqueName="19" name="LCSC#/MOUSER" queryTableFieldId="19" dataDxfId="69"/>
-    <tableColumn id="20" xr3:uid="{EEC6C7E9-C4FE-4094-B250-BB6B33BB8464}" uniqueName="20" name="Package" queryTableFieldId="20" dataDxfId="68"/>
-    <tableColumn id="21" xr3:uid="{81D33918-2986-4E3F-BD4D-051917441601}" uniqueName="21" name="Min" queryTableFieldId="21" dataDxfId="67"/>
-    <tableColumn id="22" xr3:uid="{F26EC7E1-D7C6-4ECE-B10B-99623AAEFE95}" uniqueName="22" name="Mult" queryTableFieldId="22" dataDxfId="66"/>
-    <tableColumn id="23" xr3:uid="{7AC43392-CA85-4105-977C-51ED085E626D}" uniqueName="23" name="SPQ" queryTableFieldId="23" dataDxfId="65"/>
-    <tableColumn id="24" xr3:uid="{054AEE52-D1A0-4011-B23F-BB94CFAE1142}" uniqueName="24" name="Availability" queryTableFieldId="24" dataDxfId="64"/>
-    <tableColumn id="25" xr3:uid="{0AA1D208-8245-459D-94F6-604BED0B7234}" uniqueName="25" name="Stock Status" queryTableFieldId="25" dataDxfId="63"/>
-    <tableColumn id="26" xr3:uid="{C5ABA018-08A0-4C05-B2A8-0C9FFA3C4F07}" uniqueName="26" name="Customer Notes" queryTableFieldId="26" dataDxfId="62"/>
-    <tableColumn id="27" xr3:uid="{95403B65-8FFF-446B-907D-9606ACF3E1AB}" uniqueName="27" name="Description" queryTableFieldId="27" dataDxfId="61"/>
-    <tableColumn id="28" xr3:uid="{C1157F66-0BE1-48D4-BF0E-A795DED00553}" uniqueName="28" name="Matched status" queryTableFieldId="28" dataDxfId="3"/>
-    <tableColumn id="29" xr3:uid="{B225C4F7-C17C-4475-85AA-F874BA501B03}" uniqueName="29" name="Product Link" queryTableFieldId="29" dataDxfId="2" dataCellStyle="Hyperlink 2"/>
+    <tableColumn id="9" xr3:uid="{466BF7CA-A66E-4E93-A410-26712E4A088D}" uniqueName="9" name="-" queryTableFieldId="9" dataDxfId="71"/>
+    <tableColumn id="10" xr3:uid="{EF9CED38-6BA4-4B5E-A768-E8F7877DA34C}" uniqueName="10" name="LCSC" queryTableFieldId="10" dataDxfId="70"/>
+    <tableColumn id="11" xr3:uid="{B8AF37A0-7622-4CE8-B4F8-07F8A264DAFC}" uniqueName="11" name="MOUSER" queryTableFieldId="11" dataDxfId="69"/>
+    <tableColumn id="12" xr3:uid="{3CC847EE-DB6C-4D10-A4FE-5AF7D6DAC000}" uniqueName="12" name="Already in another pcb" queryTableFieldId="12" dataDxfId="68"/>
+    <tableColumn id="13" xr3:uid="{4209E125-D2D4-4118-AAF7-2424A4EE1570}" uniqueName="13" name="--" queryTableFieldId="13" dataDxfId="67"/>
+    <tableColumn id="14" xr3:uid="{F77F0236-F98A-4965-9182-ADC25F4B7E38}" uniqueName="14" name="Mrf#" queryTableFieldId="14" dataDxfId="66"/>
+    <tableColumn id="15" xr3:uid="{35B8A93E-B4A7-4A83-9024-CC101868A70A}" uniqueName="15" name="Mfr." queryTableFieldId="15" dataDxfId="65"/>
+    <tableColumn id="16" xr3:uid="{E562ACF4-D8CD-4985-8EC9-26D45054BB92}" uniqueName="16" name="Order Qty." queryTableFieldId="16" dataDxfId="64" dataCellStyle="Currency"/>
+    <tableColumn id="17" xr3:uid="{4B8A9EA3-8B9F-48DB-B5CE-DD5C61A296C3}" uniqueName="17" name="Unit Price(USD)" queryTableFieldId="17" dataDxfId="63" dataCellStyle="Currency"/>
+    <tableColumn id="18" xr3:uid="{681F7274-0403-4F56-A317-DD049A8A07BF}" uniqueName="18" name="Ext.Price(USD)" queryTableFieldId="18" dataDxfId="62" dataCellStyle="Currency"/>
+    <tableColumn id="19" xr3:uid="{6073EC40-E9B7-4260-A82D-A28FAFFCC35E}" uniqueName="19" name="LCSC#/MOUSER" queryTableFieldId="19" dataDxfId="61"/>
+    <tableColumn id="20" xr3:uid="{EEC6C7E9-C4FE-4094-B250-BB6B33BB8464}" uniqueName="20" name="Package" queryTableFieldId="20" dataDxfId="60"/>
+    <tableColumn id="21" xr3:uid="{81D33918-2986-4E3F-BD4D-051917441601}" uniqueName="21" name="Min" queryTableFieldId="21" dataDxfId="59"/>
+    <tableColumn id="22" xr3:uid="{F26EC7E1-D7C6-4ECE-B10B-99623AAEFE95}" uniqueName="22" name="Mult" queryTableFieldId="22" dataDxfId="58"/>
+    <tableColumn id="23" xr3:uid="{7AC43392-CA85-4105-977C-51ED085E626D}" uniqueName="23" name="SPQ" queryTableFieldId="23" dataDxfId="57"/>
+    <tableColumn id="24" xr3:uid="{054AEE52-D1A0-4011-B23F-BB94CFAE1142}" uniqueName="24" name="Availability" queryTableFieldId="24" dataDxfId="56"/>
+    <tableColumn id="25" xr3:uid="{0AA1D208-8245-459D-94F6-604BED0B7234}" uniqueName="25" name="Stock Status" queryTableFieldId="25" dataDxfId="55"/>
+    <tableColumn id="26" xr3:uid="{C5ABA018-08A0-4C05-B2A8-0C9FFA3C4F07}" uniqueName="26" name="Customer Notes" queryTableFieldId="26" dataDxfId="54"/>
+    <tableColumn id="27" xr3:uid="{95403B65-8FFF-446B-907D-9606ACF3E1AB}" uniqueName="27" name="Description" queryTableFieldId="27" dataDxfId="53"/>
+    <tableColumn id="28" xr3:uid="{C1157F66-0BE1-48D4-BF0E-A795DED00553}" uniqueName="28" name="Matched status" queryTableFieldId="28" dataDxfId="52"/>
+    <tableColumn id="29" xr3:uid="{B225C4F7-C17C-4475-85AA-F874BA501B03}" uniqueName="29" name="Product Link" queryTableFieldId="29" dataDxfId="51" dataCellStyle="Hyperlink 2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -3610,34 +3593,34 @@
   </sortState>
   <tableColumns count="29">
     <tableColumn id="1" xr3:uid="{0E63F159-3CED-4B29-86B6-632E7C1C742B}" uniqueName="1" name="Id" queryTableFieldId="1"/>
-    <tableColumn id="2" xr3:uid="{D1DE625A-59DE-459D-A45A-536F2DCFBF7F}" uniqueName="2" name="Designator" queryTableFieldId="2" dataDxfId="60"/>
-    <tableColumn id="3" xr3:uid="{873A6810-3388-41FB-952D-50FC4CA27EDB}" uniqueName="3" name="Footprint" queryTableFieldId="3" dataDxfId="59"/>
+    <tableColumn id="2" xr3:uid="{D1DE625A-59DE-459D-A45A-536F2DCFBF7F}" uniqueName="2" name="Designator" queryTableFieldId="2" dataDxfId="50"/>
+    <tableColumn id="3" xr3:uid="{873A6810-3388-41FB-952D-50FC4CA27EDB}" uniqueName="3" name="Footprint" queryTableFieldId="3" dataDxfId="49"/>
     <tableColumn id="4" xr3:uid="{44B2CDFF-B5E8-4E2D-AB83-7100F24D4468}" uniqueName="4" name="Quantity" queryTableFieldId="4"/>
-    <tableColumn id="5" xr3:uid="{22FA568B-01D6-4A0C-9ECE-923A51F41F44}" uniqueName="5" name="Designation" queryTableFieldId="5" dataDxfId="58"/>
-    <tableColumn id="6" xr3:uid="{78CCE0AA-C426-48A2-9C9F-C7FD9E916E42}" uniqueName="6" name="Supplier and ref" queryTableFieldId="6" dataDxfId="57"/>
-    <tableColumn id="7" xr3:uid="{97C1A426-B683-4782-81E7-54C43CABE5DE}" uniqueName="7" name="Column1" queryTableFieldId="7" dataDxfId="56"/>
-    <tableColumn id="8" xr3:uid="{416DEE51-9BEE-4225-8B54-F5BF6C08F6B9}" uniqueName="8" name="Needed quantity" queryTableFieldId="8" dataDxfId="55"/>
-    <tableColumn id="9" xr3:uid="{32E30C7A-53F3-408B-8293-6A9B9B9AC1DF}" uniqueName="9" name="-" queryTableFieldId="9" dataDxfId="54"/>
-    <tableColumn id="10" xr3:uid="{D6C8BC49-3D09-492D-B4A4-089F31B50C42}" uniqueName="10" name="LCSC" queryTableFieldId="10" dataDxfId="53"/>
-    <tableColumn id="11" xr3:uid="{CC107E5C-29C8-4CCE-8483-88216043072D}" uniqueName="11" name="MOUSER" queryTableFieldId="11" dataDxfId="52"/>
-    <tableColumn id="12" xr3:uid="{E7EC2C75-44FB-4D79-B6F6-F9B011D6211F}" uniqueName="12" name="Already in another pcb" queryTableFieldId="12" dataDxfId="51"/>
-    <tableColumn id="13" xr3:uid="{0C385EB9-878B-4C2B-96C7-A160EB6C8B7B}" uniqueName="13" name="--" queryTableFieldId="13" dataDxfId="50"/>
-    <tableColumn id="14" xr3:uid="{D8B5CD8B-44BF-4725-BCDE-21E44EEBF205}" uniqueName="14" name="Mrf#" queryTableFieldId="14" dataDxfId="49"/>
-    <tableColumn id="15" xr3:uid="{3EF7D800-5FBD-4B86-AE11-67617320382F}" uniqueName="15" name="Mfr." queryTableFieldId="15" dataDxfId="48"/>
-    <tableColumn id="16" xr3:uid="{6D0D8B28-79C8-4C77-9563-E1F5D6B87774}" uniqueName="16" name="Order Qty." queryTableFieldId="16" dataDxfId="47" dataCellStyle="Currency"/>
-    <tableColumn id="17" xr3:uid="{4CE14486-CC74-4467-B9AD-79C240E52F93}" uniqueName="17" name="Unit Price(USD)" queryTableFieldId="17" dataDxfId="46" dataCellStyle="Currency"/>
-    <tableColumn id="18" xr3:uid="{2F6A5361-9124-455F-B3F1-383018915EB3}" uniqueName="18" name="Ext.Price(USD)" queryTableFieldId="18" dataDxfId="45" dataCellStyle="Currency"/>
-    <tableColumn id="19" xr3:uid="{78F98052-EB98-43FF-8EE5-602D557FB4D3}" uniqueName="19" name="LCSC#/MOUSER" queryTableFieldId="19" dataDxfId="44"/>
-    <tableColumn id="20" xr3:uid="{4F449396-32DC-4534-BFE5-AA61E6C0DC5A}" uniqueName="20" name="Package" queryTableFieldId="20" dataDxfId="43"/>
-    <tableColumn id="21" xr3:uid="{26D2A300-326B-49F5-84C9-02EB05291F90}" uniqueName="21" name="Min" queryTableFieldId="21" dataDxfId="42"/>
-    <tableColumn id="22" xr3:uid="{5CAF8612-E695-4A48-836A-F8A9EDFB3CB8}" uniqueName="22" name="Mult" queryTableFieldId="22" dataDxfId="41"/>
-    <tableColumn id="23" xr3:uid="{9A05AEF9-585A-4855-B11C-CAE738DD58FA}" uniqueName="23" name="SPQ" queryTableFieldId="23" dataDxfId="40"/>
-    <tableColumn id="24" xr3:uid="{3D7F11A3-37D2-4805-AEBA-B9E26E5E28E9}" uniqueName="24" name="Availability" queryTableFieldId="24" dataDxfId="39"/>
-    <tableColumn id="25" xr3:uid="{933DBD96-9E4F-43F7-A800-CD83B0A44E24}" uniqueName="25" name="Stock Status" queryTableFieldId="25" dataDxfId="38"/>
-    <tableColumn id="26" xr3:uid="{32899468-D5AC-4CCC-BF0C-B9A3CB2B5492}" uniqueName="26" name="Customer Notes" queryTableFieldId="26" dataDxfId="37"/>
-    <tableColumn id="27" xr3:uid="{8CDB5DD7-778C-4CF7-A3C5-BE2C00EB1D37}" uniqueName="27" name="Description" queryTableFieldId="27" dataDxfId="36"/>
-    <tableColumn id="28" xr3:uid="{F1DA22D8-5468-4D00-B4F4-CB4FD27BE53B}" uniqueName="28" name="Matched status" queryTableFieldId="28" dataDxfId="1"/>
-    <tableColumn id="29" xr3:uid="{687D4C7B-94A2-47A4-BECA-516084FF4352}" uniqueName="29" name="Product Link" queryTableFieldId="29" dataDxfId="0" dataCellStyle="Hyperlink 2"/>
+    <tableColumn id="5" xr3:uid="{22FA568B-01D6-4A0C-9ECE-923A51F41F44}" uniqueName="5" name="Designation" queryTableFieldId="5" dataDxfId="48"/>
+    <tableColumn id="6" xr3:uid="{78CCE0AA-C426-48A2-9C9F-C7FD9E916E42}" uniqueName="6" name="Supplier and ref" queryTableFieldId="6" dataDxfId="47"/>
+    <tableColumn id="7" xr3:uid="{97C1A426-B683-4782-81E7-54C43CABE5DE}" uniqueName="7" name="Column1" queryTableFieldId="7" dataDxfId="46"/>
+    <tableColumn id="8" xr3:uid="{416DEE51-9BEE-4225-8B54-F5BF6C08F6B9}" uniqueName="8" name="Needed quantity" queryTableFieldId="8" dataDxfId="45"/>
+    <tableColumn id="9" xr3:uid="{32E30C7A-53F3-408B-8293-6A9B9B9AC1DF}" uniqueName="9" name="-" queryTableFieldId="9" dataDxfId="44"/>
+    <tableColumn id="10" xr3:uid="{D6C8BC49-3D09-492D-B4A4-089F31B50C42}" uniqueName="10" name="LCSC" queryTableFieldId="10" dataDxfId="43"/>
+    <tableColumn id="11" xr3:uid="{CC107E5C-29C8-4CCE-8483-88216043072D}" uniqueName="11" name="MOUSER" queryTableFieldId="11" dataDxfId="42"/>
+    <tableColumn id="12" xr3:uid="{E7EC2C75-44FB-4D79-B6F6-F9B011D6211F}" uniqueName="12" name="Already in another pcb" queryTableFieldId="12" dataDxfId="41"/>
+    <tableColumn id="13" xr3:uid="{0C385EB9-878B-4C2B-96C7-A160EB6C8B7B}" uniqueName="13" name="--" queryTableFieldId="13" dataDxfId="40"/>
+    <tableColumn id="14" xr3:uid="{D8B5CD8B-44BF-4725-BCDE-21E44EEBF205}" uniqueName="14" name="Mrf#" queryTableFieldId="14" dataDxfId="39"/>
+    <tableColumn id="15" xr3:uid="{3EF7D800-5FBD-4B86-AE11-67617320382F}" uniqueName="15" name="Mfr." queryTableFieldId="15" dataDxfId="38"/>
+    <tableColumn id="16" xr3:uid="{6D0D8B28-79C8-4C77-9563-E1F5D6B87774}" uniqueName="16" name="Order Qty." queryTableFieldId="16" dataDxfId="37" dataCellStyle="Currency"/>
+    <tableColumn id="17" xr3:uid="{4CE14486-CC74-4467-B9AD-79C240E52F93}" uniqueName="17" name="Unit Price(USD)" queryTableFieldId="17" dataDxfId="36" dataCellStyle="Currency"/>
+    <tableColumn id="18" xr3:uid="{2F6A5361-9124-455F-B3F1-383018915EB3}" uniqueName="18" name="Ext.Price(USD)" queryTableFieldId="18" dataDxfId="35" dataCellStyle="Currency"/>
+    <tableColumn id="19" xr3:uid="{78F98052-EB98-43FF-8EE5-602D557FB4D3}" uniqueName="19" name="LCSC#/MOUSER" queryTableFieldId="19" dataDxfId="34"/>
+    <tableColumn id="20" xr3:uid="{4F449396-32DC-4534-BFE5-AA61E6C0DC5A}" uniqueName="20" name="Package" queryTableFieldId="20" dataDxfId="33"/>
+    <tableColumn id="21" xr3:uid="{26D2A300-326B-49F5-84C9-02EB05291F90}" uniqueName="21" name="Min" queryTableFieldId="21" dataDxfId="32"/>
+    <tableColumn id="22" xr3:uid="{5CAF8612-E695-4A48-836A-F8A9EDFB3CB8}" uniqueName="22" name="Mult" queryTableFieldId="22" dataDxfId="31"/>
+    <tableColumn id="23" xr3:uid="{9A05AEF9-585A-4855-B11C-CAE738DD58FA}" uniqueName="23" name="SPQ" queryTableFieldId="23" dataDxfId="30"/>
+    <tableColumn id="24" xr3:uid="{3D7F11A3-37D2-4805-AEBA-B9E26E5E28E9}" uniqueName="24" name="Availability" queryTableFieldId="24" dataDxfId="29"/>
+    <tableColumn id="25" xr3:uid="{933DBD96-9E4F-43F7-A800-CD83B0A44E24}" uniqueName="25" name="Stock Status" queryTableFieldId="25" dataDxfId="28"/>
+    <tableColumn id="26" xr3:uid="{32899468-D5AC-4CCC-BF0C-B9A3CB2B5492}" uniqueName="26" name="Customer Notes" queryTableFieldId="26" dataDxfId="27"/>
+    <tableColumn id="27" xr3:uid="{8CDB5DD7-778C-4CF7-A3C5-BE2C00EB1D37}" uniqueName="27" name="Description" queryTableFieldId="27" dataDxfId="26"/>
+    <tableColumn id="28" xr3:uid="{F1DA22D8-5468-4D00-B4F4-CB4FD27BE53B}" uniqueName="28" name="Matched status" queryTableFieldId="28" dataDxfId="25"/>
+    <tableColumn id="29" xr3:uid="{687D4C7B-94A2-47A4-BECA-516084FF4352}" uniqueName="29" name="Product Link" queryTableFieldId="29" dataDxfId="24" dataCellStyle="Hyperlink 2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -3648,12 +3631,12 @@
   <autoFilter ref="A1:G10" xr:uid="{358C07D9-C534-4C2D-B737-344400F670C4}"/>
   <tableColumns count="7">
     <tableColumn id="1" xr3:uid="{0F19A646-43F4-4862-8B93-9080417C7268}" uniqueName="1" name="Id" queryTableFieldId="1"/>
-    <tableColumn id="2" xr3:uid="{7198E0C1-4967-4BBD-9D55-A70B2A61C192}" uniqueName="2" name="Designator" queryTableFieldId="2" dataDxfId="35"/>
-    <tableColumn id="3" xr3:uid="{C2A2451A-0F59-404F-AA66-0DD98A96CB6B}" uniqueName="3" name="Footprint" queryTableFieldId="3" dataDxfId="34"/>
+    <tableColumn id="2" xr3:uid="{7198E0C1-4967-4BBD-9D55-A70B2A61C192}" uniqueName="2" name="Designator" queryTableFieldId="2" dataDxfId="23"/>
+    <tableColumn id="3" xr3:uid="{C2A2451A-0F59-404F-AA66-0DD98A96CB6B}" uniqueName="3" name="Footprint" queryTableFieldId="3" dataDxfId="22"/>
     <tableColumn id="4" xr3:uid="{57EDD4F3-19D9-42B5-A4D4-17B50797C919}" uniqueName="4" name="Quantity" queryTableFieldId="4"/>
-    <tableColumn id="5" xr3:uid="{AC6AFA26-0E57-46AC-BB98-3942162B3F06}" uniqueName="5" name="Designation" queryTableFieldId="5" dataDxfId="33"/>
-    <tableColumn id="6" xr3:uid="{3285DEC9-31B3-4F44-B1AD-0B3851AF39BA}" uniqueName="6" name="Supplier and ref" queryTableFieldId="6" dataDxfId="32"/>
-    <tableColumn id="7" xr3:uid="{AA28C35C-D1F9-457B-A91B-14B4A9A05C17}" uniqueName="7" name="Column1" queryTableFieldId="7" dataDxfId="31"/>
+    <tableColumn id="5" xr3:uid="{AC6AFA26-0E57-46AC-BB98-3942162B3F06}" uniqueName="5" name="Designation" queryTableFieldId="5" dataDxfId="21"/>
+    <tableColumn id="6" xr3:uid="{3285DEC9-31B3-4F44-B1AD-0B3851AF39BA}" uniqueName="6" name="Supplier and ref" queryTableFieldId="6" dataDxfId="20"/>
+    <tableColumn id="7" xr3:uid="{AA28C35C-D1F9-457B-A91B-14B4A9A05C17}" uniqueName="7" name="Column1" queryTableFieldId="7" dataDxfId="19"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -3667,19 +3650,19 @@
   </sortState>
   <tableColumns count="12">
     <tableColumn id="1" xr3:uid="{ADE8F525-CFD6-41FB-A869-878D887125F2}" uniqueName="1" name="Id" queryTableFieldId="1"/>
-    <tableColumn id="2" xr3:uid="{06802B0A-38DB-4939-98FE-D825FBBCF621}" uniqueName="2" name="Designator" queryTableFieldId="2" dataDxfId="30"/>
-    <tableColumn id="3" xr3:uid="{A0E49D32-4602-4A36-A99A-61255BE52689}" uniqueName="3" name="Footprint" queryTableFieldId="3" dataDxfId="29"/>
+    <tableColumn id="2" xr3:uid="{06802B0A-38DB-4939-98FE-D825FBBCF621}" uniqueName="2" name="Designator" queryTableFieldId="2" dataDxfId="18"/>
+    <tableColumn id="3" xr3:uid="{A0E49D32-4602-4A36-A99A-61255BE52689}" uniqueName="3" name="Footprint" queryTableFieldId="3" dataDxfId="17"/>
     <tableColumn id="4" xr3:uid="{2639D562-1AB7-4369-9C38-6DE58E9DE4E0}" uniqueName="4" name="Quantity" queryTableFieldId="4"/>
-    <tableColumn id="5" xr3:uid="{E918130A-210D-4D0D-B354-0424657F3D8A}" uniqueName="5" name="Designation" queryTableFieldId="5" dataDxfId="28"/>
-    <tableColumn id="6" xr3:uid="{2852533A-8BB7-4324-9C65-B20AD7F9634F}" uniqueName="6" name="Supplier and ref" queryTableFieldId="6" dataDxfId="27"/>
-    <tableColumn id="7" xr3:uid="{FCD08B98-7123-4ED3-95E6-F7165F6496EF}" uniqueName="7" name="Column1" queryTableFieldId="7" dataDxfId="26"/>
-    <tableColumn id="10" xr3:uid="{D704FAE8-15F6-48B1-9F78-ECE42633C6A6}" uniqueName="10" name="Needed quantity" queryTableFieldId="9" dataDxfId="25">
+    <tableColumn id="5" xr3:uid="{E918130A-210D-4D0D-B354-0424657F3D8A}" uniqueName="5" name="Designation" queryTableFieldId="5" dataDxfId="16"/>
+    <tableColumn id="6" xr3:uid="{2852533A-8BB7-4324-9C65-B20AD7F9634F}" uniqueName="6" name="Supplier and ref" queryTableFieldId="6" dataDxfId="15"/>
+    <tableColumn id="7" xr3:uid="{FCD08B98-7123-4ED3-95E6-F7165F6496EF}" uniqueName="7" name="Column1" queryTableFieldId="7" dataDxfId="14"/>
+    <tableColumn id="10" xr3:uid="{D704FAE8-15F6-48B1-9F78-ECE42633C6A6}" uniqueName="10" name="Needed quantity" queryTableFieldId="9" dataDxfId="13">
       <calculatedColumnFormula>2*Artnet_DMX_Converter[[#This Row],[Quantity]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{912033B7-820A-4CB4-A444-84EA4F66B927}" uniqueName="8" name="_1" queryTableFieldId="8" dataDxfId="24"/>
-    <tableColumn id="11" xr3:uid="{D185F272-ECD8-4D0C-A8C0-5C517F5CB2C3}" uniqueName="11" name="Column12" queryTableFieldId="10" dataDxfId="23"/>
-    <tableColumn id="12" xr3:uid="{8235DE14-4219-4B94-81A0-74DA669B2200}" uniqueName="12" name="Column13" queryTableFieldId="11" dataDxfId="22"/>
-    <tableColumn id="13" xr3:uid="{0CB54720-3FD3-41A1-B176-167D3F8B9C1F}" uniqueName="13" name="Column14" queryTableFieldId="12" dataDxfId="21"/>
+    <tableColumn id="8" xr3:uid="{912033B7-820A-4CB4-A444-84EA4F66B927}" uniqueName="8" name="_1" queryTableFieldId="8" dataDxfId="12"/>
+    <tableColumn id="11" xr3:uid="{D185F272-ECD8-4D0C-A8C0-5C517F5CB2C3}" uniqueName="11" name="Column12" queryTableFieldId="10" dataDxfId="11"/>
+    <tableColumn id="12" xr3:uid="{8235DE14-4219-4B94-81A0-74DA669B2200}" uniqueName="12" name="Column13" queryTableFieldId="11" dataDxfId="10"/>
+    <tableColumn id="13" xr3:uid="{0CB54720-3FD3-41A1-B176-167D3F8B9C1F}" uniqueName="13" name="Column14" queryTableFieldId="12" dataDxfId="9"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -3690,13 +3673,13 @@
   <autoFilter ref="A1:H12" xr:uid="{7769F78E-5E6C-4F2E-A421-D9864D32DBFF}"/>
   <tableColumns count="8">
     <tableColumn id="1" xr3:uid="{BEBDD4F5-047E-42EE-AF7A-AEC96CC412EB}" uniqueName="1" name="Id" queryTableFieldId="1"/>
-    <tableColumn id="2" xr3:uid="{70C04B8F-9B5D-4AE8-811E-7A325F5B3B32}" uniqueName="2" name="Designator" queryTableFieldId="2" dataDxfId="20"/>
-    <tableColumn id="3" xr3:uid="{5D3B3C5B-89C3-4145-BEFA-49CD552602EC}" uniqueName="3" name="Footprint" queryTableFieldId="3" dataDxfId="19"/>
+    <tableColumn id="2" xr3:uid="{70C04B8F-9B5D-4AE8-811E-7A325F5B3B32}" uniqueName="2" name="Designator" queryTableFieldId="2" dataDxfId="8"/>
+    <tableColumn id="3" xr3:uid="{5D3B3C5B-89C3-4145-BEFA-49CD552602EC}" uniqueName="3" name="Footprint" queryTableFieldId="3" dataDxfId="7"/>
     <tableColumn id="4" xr3:uid="{C6D2277C-C53C-42BD-B1B1-3F5BD927522F}" uniqueName="4" name="Quantity" queryTableFieldId="4"/>
-    <tableColumn id="5" xr3:uid="{50C12BFC-08EC-4014-8DE1-7360FE30FFEE}" uniqueName="5" name="Designation" queryTableFieldId="5" dataDxfId="18"/>
-    <tableColumn id="6" xr3:uid="{5E872B7B-44C6-474C-8EE6-2996F8257863}" uniqueName="6" name="Supplier and ref" queryTableFieldId="6" dataDxfId="17"/>
-    <tableColumn id="7" xr3:uid="{8616BBA3-0AE5-4D84-BE4F-A09C69812E1F}" uniqueName="7" name="Column1" queryTableFieldId="7" dataDxfId="16"/>
-    <tableColumn id="8" xr3:uid="{83C5AA2C-C2E2-4E7E-82D8-7C221C32DC65}" uniqueName="8" name="_1" queryTableFieldId="8" dataDxfId="15"/>
+    <tableColumn id="5" xr3:uid="{50C12BFC-08EC-4014-8DE1-7360FE30FFEE}" uniqueName="5" name="Designation" queryTableFieldId="5" dataDxfId="6"/>
+    <tableColumn id="6" xr3:uid="{5E872B7B-44C6-474C-8EE6-2996F8257863}" uniqueName="6" name="Supplier and ref" queryTableFieldId="6" dataDxfId="5"/>
+    <tableColumn id="7" xr3:uid="{8616BBA3-0AE5-4D84-BE4F-A09C69812E1F}" uniqueName="7" name="Column1" queryTableFieldId="7" dataDxfId="4"/>
+    <tableColumn id="8" xr3:uid="{83C5AA2C-C2E2-4E7E-82D8-7C221C32DC65}" uniqueName="8" name="_1" queryTableFieldId="8" dataDxfId="3"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -4019,7 +4002,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{77A293D4-B4DA-4789-A163-7A7FEBE93979}">
-  <dimension ref="A1:AV116"/>
+  <dimension ref="A1:AV122"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="18" customWidth="1"/>
@@ -4039,7 +4022,7 @@
     <col min="26" max="26" width="9.140625" style="14"/>
     <col min="27" max="27" width="43.28515625" style="14" customWidth="1"/>
     <col min="28" max="28" width="9.140625" style="14"/>
-    <col min="29" max="29" width="104.5703125" style="24" customWidth="1"/>
+    <col min="29" max="29" width="104.5703125" style="14" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:29" ht="15" customHeight="1">
@@ -6316,7 +6299,7 @@
       <c r="S29" s="17" t="s">
         <v>624</v>
       </c>
-      <c r="AC29" s="26" t="s">
+      <c r="AC29" s="25" t="s">
         <v>639</v>
       </c>
     </row>
@@ -6686,7 +6669,7 @@
       <c r="S34" s="14" t="s">
         <v>627</v>
       </c>
-      <c r="AC34" s="26" t="s">
+      <c r="AC34" s="25" t="s">
         <v>640</v>
       </c>
     </row>
@@ -6739,7 +6722,7 @@
       <c r="S35" s="14" t="s">
         <v>630</v>
       </c>
-      <c r="AC35" s="26" t="s">
+      <c r="AC35" s="25" t="s">
         <v>641</v>
       </c>
     </row>
@@ -6792,7 +6775,7 @@
       <c r="S36" s="14" t="s">
         <v>631</v>
       </c>
-      <c r="AC36" s="26" t="s">
+      <c r="AC36" s="25" t="s">
         <v>642</v>
       </c>
     </row>
@@ -7594,7 +7577,7 @@
       <c r="AB46" t="s">
         <v>235</v>
       </c>
-      <c r="AC46" s="26" t="s">
+      <c r="AC46" s="25" t="s">
         <v>649</v>
       </c>
     </row>
@@ -8677,7 +8660,7 @@
       <c r="S60" s="14" t="s">
         <v>632</v>
       </c>
-      <c r="AC60" s="26" t="s">
+      <c r="AC60" s="25" t="s">
         <v>643</v>
       </c>
       <c r="AN60" s="4"/>
@@ -8972,7 +8955,7 @@
       <c r="S64" s="14" t="s">
         <v>633</v>
       </c>
-      <c r="AC64" s="26" t="s">
+      <c r="AC64" s="25" t="s">
         <v>644</v>
       </c>
       <c r="AN64" s="4"/>
@@ -9027,7 +9010,7 @@
       <c r="S65" s="14" t="s">
         <v>636</v>
       </c>
-      <c r="AC65" s="26" t="s">
+      <c r="AC65" s="25" t="s">
         <v>645</v>
       </c>
     </row>
@@ -9838,7 +9821,7 @@
       <c r="Z77" s="22"/>
       <c r="AA77" s="22"/>
       <c r="AB77"/>
-      <c r="AC77" s="25"/>
+      <c r="AC77" s="24"/>
     </row>
     <row r="78" spans="1:29" ht="15" customHeight="1">
       <c r="A78" t="s">
@@ -9959,7 +9942,7 @@
         <v>186</v>
       </c>
       <c r="P79" s="18"/>
-      <c r="AC79" s="27"/>
+      <c r="AC79" s="26"/>
     </row>
     <row r="80" spans="1:29" ht="15" customHeight="1">
       <c r="A80">
@@ -9991,7 +9974,7 @@
         <v>186</v>
       </c>
       <c r="P80" s="18"/>
-      <c r="AC80" s="27"/>
+      <c r="AC80" s="26"/>
     </row>
     <row r="81" spans="1:29" ht="15" customHeight="1">
       <c r="A81">
@@ -10099,7 +10082,7 @@
         <v>186</v>
       </c>
       <c r="P82" s="18"/>
-      <c r="AC82" s="27"/>
+      <c r="AC82" s="26"/>
     </row>
     <row r="83" spans="1:29" ht="15" customHeight="1">
       <c r="A83">
@@ -10207,7 +10190,7 @@
         <v>186</v>
       </c>
       <c r="P84" s="18"/>
-      <c r="AC84" s="27"/>
+      <c r="AC84" s="26"/>
     </row>
     <row r="85" spans="1:29" ht="15" customHeight="1">
       <c r="A85">
@@ -10239,7 +10222,7 @@
         <v>186</v>
       </c>
       <c r="P85" s="18"/>
-      <c r="AC85" s="27"/>
+      <c r="AC85" s="26"/>
     </row>
     <row r="86" spans="1:29" ht="15" customHeight="1">
       <c r="A86">
@@ -10670,7 +10653,7 @@
         <v>186</v>
       </c>
       <c r="P93" s="18"/>
-      <c r="AC93" s="27"/>
+      <c r="AC93" s="26"/>
     </row>
     <row r="94" spans="1:29" ht="15" customHeight="1">
       <c r="A94">
@@ -11079,7 +11062,7 @@
         <v>4</v>
       </c>
       <c r="P99" s="18"/>
-      <c r="AC99" s="27"/>
+      <c r="AC99" s="26"/>
     </row>
     <row r="100" spans="1:29" ht="15" customHeight="1">
       <c r="A100">
@@ -11232,20 +11215,20 @@
     </row>
     <row r="102" spans="1:29" ht="15" customHeight="1">
       <c r="P102" s="18"/>
-      <c r="AC102" s="27"/>
+      <c r="AC102" s="26"/>
     </row>
     <row r="103" spans="1:29" ht="15" customHeight="1">
       <c r="P103" s="18"/>
-      <c r="AC103" s="27"/>
+      <c r="AC103" s="26"/>
     </row>
     <row r="104" spans="1:29" ht="15" customHeight="1">
       <c r="O104" s="20"/>
       <c r="P104" s="18"/>
-      <c r="AC104" s="27"/>
+      <c r="AC104" s="26"/>
     </row>
     <row r="105" spans="1:29" ht="15" customHeight="1">
       <c r="P105" s="18"/>
-      <c r="AC105" s="27"/>
+      <c r="AC105" s="26"/>
     </row>
     <row r="106" spans="1:29" ht="15" customHeight="1">
       <c r="A106" t="s">
@@ -11313,7 +11296,7 @@
       <c r="AB106" s="9" t="s">
         <v>235</v>
       </c>
-      <c r="AC106" s="26" t="s">
+      <c r="AC106" s="25" t="s">
         <v>529</v>
       </c>
     </row>
@@ -11382,7 +11365,7 @@
       <c r="AB107" s="9" t="s">
         <v>235</v>
       </c>
-      <c r="AC107" s="26" t="s">
+      <c r="AC107" s="25" t="s">
         <v>599</v>
       </c>
     </row>
@@ -11412,33 +11395,90 @@
       <c r="AA108" t="s">
         <v>652</v>
       </c>
-      <c r="AC108" s="27" t="s">
+      <c r="AC108" s="26" t="s">
         <v>654</v>
       </c>
     </row>
     <row r="109" spans="1:29" ht="15" customHeight="1"/>
     <row r="110" spans="1:29" ht="15" customHeight="1"/>
-    <row r="111" spans="1:29" ht="15" customHeight="1"/>
-    <row r="112" spans="1:29" ht="15" customHeight="1"/>
-    <row r="113" spans="18:18" ht="15" customHeight="1"/>
-    <row r="114" spans="18:18" ht="15" customHeight="1">
-      <c r="R114" s="19">
-        <f>SUM(Artnet_DMX_Converter5[Ext.Price(USD)],Display_panel7[Ext.Price(USD)],WIFI_Module9[Ext.Price(USD)],R104:R113)</f>
-        <v>206.52000000000004</v>
-      </c>
-    </row>
-    <row r="115" spans="18:18" ht="15" customHeight="1"/>
-    <row r="116" spans="18:18" ht="15" customHeight="1"/>
+    <row r="111" spans="1:29" ht="15" customHeight="1">
+      <c r="N111" s="14" t="s">
+        <v>660</v>
+      </c>
+      <c r="R111" s="19">
+        <v>14.11</v>
+      </c>
+    </row>
+    <row r="112" spans="1:29" ht="15" customHeight="1">
+      <c r="N112" s="14" t="s">
+        <v>661</v>
+      </c>
+      <c r="R112" s="19">
+        <v>5.05</v>
+      </c>
+    </row>
+    <row r="113" spans="14:19" ht="15" customHeight="1">
+      <c r="N113" s="14" t="s">
+        <v>662</v>
+      </c>
+      <c r="R113" s="19">
+        <v>7.05</v>
+      </c>
+      <c r="S113" s="28"/>
+    </row>
+    <row r="114" spans="14:19" ht="15" customHeight="1"/>
+    <row r="115" spans="14:19" ht="15" customHeight="1"/>
+    <row r="116" spans="14:19" ht="15" customHeight="1">
+      <c r="N116" s="14" t="s">
+        <v>655</v>
+      </c>
+      <c r="R116" s="27">
+        <v>14.87</v>
+      </c>
+    </row>
+    <row r="117" spans="14:19">
+      <c r="N117" s="14" t="s">
+        <v>656</v>
+      </c>
+      <c r="R117" s="27">
+        <v>14.89</v>
+      </c>
+    </row>
+    <row r="118" spans="14:19">
+      <c r="N118" s="14" t="s">
+        <v>657</v>
+      </c>
+      <c r="R118" s="19">
+        <v>6.9</v>
+      </c>
+    </row>
+    <row r="119" spans="14:19">
+      <c r="N119" s="14" t="s">
+        <v>658</v>
+      </c>
+      <c r="R119" s="19">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="122" spans="14:19">
+      <c r="N122" s="14" t="s">
+        <v>659</v>
+      </c>
+      <c r="R122" s="19">
+        <f>SUM(Artnet_DMX_Converter5[Ext.Price(USD)],Display_panel7[Ext.Price(USD)],WIFI_Module9[Ext.Price(USD)],R104:R119)</f>
+        <v>269.39000000000004</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <conditionalFormatting sqref="M2:M108">
-    <cfRule type="expression" dxfId="14" priority="1">
+    <cfRule type="expression" dxfId="2" priority="1">
       <formula>P2&gt;H2</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="13" priority="2">
+    <cfRule type="expression" dxfId="1" priority="2">
       <formula>P2=H2</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="12" priority="3">
+    <cfRule type="expression" dxfId="0" priority="3">
       <formula>P2&lt;H2</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>